<commit_message>
still working on verify all data in input file to what is in the pcp system; removed tab name, eg "memebership::" from field name checks since they are not needed when importing at all.
</commit_message>
<xml_diff>
--- a/pcp_realm_inport_export/pcp_realm_map.xlsx
+++ b/pcp_realm_inport_export/pcp_realm_map.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Denise/Library/CloudStorage/Dropbox/4thU/process_automations/pcp_to_cc_root/pcp_realm_inport_export/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C40C53A1-15B7-3C44-86A2-989508FAA124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC059D6-88C3-9F44-9357-6CFEC971434F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2900" yWindow="2560" windowWidth="26260" windowHeight="15640" xr2:uid="{6517D458-34DE-0A49-98D4-48FE74C8A8ED}"/>
+    <workbookView xWindow="1980" yWindow="1120" windowWidth="26260" windowHeight="15640" xr2:uid="{6517D458-34DE-0A49-98D4-48FE74C8A8ED}"/>
   </bookViews>
   <sheets>
     <sheet name="columns" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">columns!$A$1:$J$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">columns!$A$1:$K$92</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="136">
   <si>
     <t>x</t>
   </si>
@@ -440,13 +440,13 @@
     <t>pcp_relation_to_4thu</t>
   </si>
   <si>
-    <t>Realm Field::Languages Spoken</t>
-  </si>
-  <si>
     <t>Realm Field::Member Status</t>
   </si>
   <si>
-    <t>Realm Field::Date Joined Fourth U</t>
+    <t>pcp_field_type</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
 </sst>
 </file>
@@ -825,22 +825,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{010D235E-A6DF-7F4E-844A-20CA78631965}">
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:M92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="29.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.1640625" customWidth="1"/>
+    <col min="6" max="6" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>122</v>
       </c>
@@ -854,31 +855,34 @@
         <v>123</v>
       </c>
       <c r="E1" t="s">
+        <v>134</v>
+      </c>
+      <c r="F1" t="s">
         <v>119</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>118</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>124</v>
       </c>
-      <c r="H1" t="s">
-        <v>0</v>
-      </c>
       <c r="I1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" t="s">
         <v>117</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>116</v>
       </c>
-      <c r="K1" t="s">
-        <v>0</v>
-      </c>
       <c r="L1" t="s">
+        <v>0</v>
+      </c>
+      <c r="M1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>114</v>
       </c>
@@ -888,20 +892,20 @@
       <c r="C2" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>113</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>1</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>112</v>
       </c>
@@ -911,40 +915,38 @@
       <c r="C3" t="s">
         <v>0</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>111</v>
       </c>
-      <c r="F3" t="s">
-        <v>0</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="G3" s="1"/>
+      <c r="J3" t="s">
         <v>111</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>3</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>110</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>109</v>
       </c>
-      <c r="J4">
+      <c r="K4">
         <v>4</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>109</v>
       </c>
@@ -954,60 +956,54 @@
       <c r="C5" t="s">
         <v>0</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>109</v>
       </c>
-      <c r="F5" t="s">
-        <v>0</v>
-      </c>
-      <c r="I5" t="s">
+      <c r="G5" s="1"/>
+      <c r="J5" t="s">
         <v>107</v>
       </c>
-      <c r="J5">
+      <c r="K5">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>108</v>
       </c>
       <c r="B6">
         <v>6</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>106</v>
       </c>
-      <c r="F6" t="s">
-        <v>0</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="G6" s="1"/>
+      <c r="J6" t="s">
         <v>105</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>107</v>
       </c>
       <c r="B7">
         <v>7</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>107</v>
       </c>
-      <c r="F7" t="s">
-        <v>0</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="G7" s="1"/>
+      <c r="J7" t="s">
         <v>103</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>105</v>
       </c>
@@ -1017,20 +1013,18 @@
       <c r="C8" t="s">
         <v>0</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>105</v>
       </c>
-      <c r="F8" t="s">
-        <v>0</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="G8" s="1"/>
+      <c r="J8" t="s">
         <v>106</v>
       </c>
-      <c r="J8">
+      <c r="K8">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>104</v>
       </c>
@@ -1043,20 +1037,18 @@
       <c r="D9" t="s">
         <v>0</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>103</v>
       </c>
-      <c r="F9" t="s">
-        <v>0</v>
-      </c>
-      <c r="I9" t="s">
+      <c r="G9" s="1"/>
+      <c r="J9" t="s">
         <v>80</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>88</v>
       </c>
@@ -1066,20 +1058,18 @@
       <c r="D10" t="s">
         <v>0</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>88</v>
       </c>
-      <c r="F10" t="s">
-        <v>0</v>
-      </c>
-      <c r="I10" t="s">
+      <c r="G10" s="1"/>
+      <c r="J10" t="s">
         <v>77</v>
       </c>
-      <c r="J10">
+      <c r="K10">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>102</v>
       </c>
@@ -1089,34 +1079,32 @@
       <c r="D11" t="s">
         <v>0</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>75</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>82</v>
       </c>
       <c r="B12">
         <v>12</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>82</v>
       </c>
-      <c r="F12" t="s">
-        <v>0</v>
-      </c>
-      <c r="I12" t="s">
+      <c r="G12" s="1"/>
+      <c r="J12" t="s">
         <v>72</v>
       </c>
-      <c r="J12">
+      <c r="K12">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>101</v>
       </c>
@@ -1126,14 +1114,14 @@
       <c r="D13" t="s">
         <v>0</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>125</v>
       </c>
-      <c r="J13">
+      <c r="K13">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>100</v>
       </c>
@@ -1143,14 +1131,14 @@
       <c r="D14" t="s">
         <v>0</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>66</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>99</v>
       </c>
@@ -1160,14 +1148,14 @@
       <c r="D15" t="s">
         <v>0</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>57</v>
       </c>
-      <c r="J15">
+      <c r="K15">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>98</v>
       </c>
@@ -1177,48 +1165,46 @@
       <c r="D16" t="s">
         <v>0</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>55</v>
       </c>
-      <c r="J16">
+      <c r="K16">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>84</v>
       </c>
       <c r="B17">
         <v>17</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="F17" t="s">
-        <v>0</v>
-      </c>
-      <c r="I17" t="s">
+      <c r="G17" s="1"/>
+      <c r="J17" t="s">
         <v>53</v>
       </c>
-      <c r="J17">
+      <c r="K17">
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>97</v>
       </c>
       <c r="B18">
         <v>18</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>51</v>
       </c>
-      <c r="J18">
+      <c r="K18">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>96</v>
       </c>
@@ -1231,14 +1217,14 @@
       <c r="D19" t="s">
         <v>0</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>49</v>
       </c>
-      <c r="J19">
+      <c r="K19">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>95</v>
       </c>
@@ -1248,14 +1234,14 @@
       <c r="D20" t="s">
         <v>0</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>46</v>
       </c>
-      <c r="J20">
+      <c r="K20">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>94</v>
       </c>
@@ -1265,112 +1251,112 @@
       <c r="D21" t="s">
         <v>0</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>42</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>93</v>
       </c>
       <c r="B22">
         <v>22</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>44</v>
       </c>
-      <c r="J22">
+      <c r="K22">
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>92</v>
       </c>
       <c r="B23">
         <v>23</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>40</v>
       </c>
-      <c r="J23">
+      <c r="K23">
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>91</v>
       </c>
       <c r="B24">
         <v>24</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>35</v>
       </c>
-      <c r="J24">
+      <c r="K24">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>90</v>
       </c>
       <c r="B25">
         <v>25</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>33</v>
       </c>
-      <c r="J25">
+      <c r="K25">
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>89</v>
       </c>
       <c r="B26">
         <v>26</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" t="s">
         <v>31</v>
       </c>
-      <c r="J26">
+      <c r="K26">
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>87</v>
       </c>
       <c r="B27">
         <v>27</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>88</v>
       </c>
-      <c r="J27">
+      <c r="K27">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>85</v>
       </c>
       <c r="B28">
         <v>28</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>86</v>
       </c>
-      <c r="J28">
+      <c r="K28">
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>83</v>
       </c>
@@ -1380,14 +1366,14 @@
       <c r="D29" t="s">
         <v>0</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>84</v>
       </c>
-      <c r="J29">
+      <c r="K29">
         <v>29</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>81</v>
       </c>
@@ -1397,20 +1383,18 @@
       <c r="D30" t="s">
         <v>0</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>80</v>
       </c>
-      <c r="F30" t="s">
-        <v>0</v>
-      </c>
-      <c r="I30" t="s">
+      <c r="G30" s="1"/>
+      <c r="J30" t="s">
         <v>82</v>
       </c>
-      <c r="J30">
+      <c r="K30">
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>78</v>
       </c>
@@ -1420,20 +1404,18 @@
       <c r="D31" t="s">
         <v>0</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F31" t="s">
         <v>77</v>
       </c>
-      <c r="F31" t="s">
-        <v>0</v>
-      </c>
-      <c r="I31" t="s">
+      <c r="G31" s="1"/>
+      <c r="J31" t="s">
         <v>79</v>
       </c>
-      <c r="J31">
+      <c r="K31">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>76</v>
       </c>
@@ -1443,20 +1425,18 @@
       <c r="D32" t="s">
         <v>0</v>
       </c>
-      <c r="E32" t="s">
+      <c r="F32" t="s">
         <v>75</v>
       </c>
-      <c r="F32" t="s">
-        <v>0</v>
-      </c>
-      <c r="I32" t="s">
+      <c r="G32" s="1"/>
+      <c r="J32" t="s">
         <v>1</v>
       </c>
-      <c r="J32">
+      <c r="K32">
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>73</v>
       </c>
@@ -1466,20 +1446,18 @@
       <c r="D33" t="s">
         <v>0</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>72</v>
       </c>
-      <c r="F33" t="s">
-        <v>0</v>
-      </c>
-      <c r="I33" t="s">
+      <c r="G33" s="1"/>
+      <c r="J33" t="s">
         <v>74</v>
       </c>
-      <c r="J33">
+      <c r="K33">
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>70</v>
       </c>
@@ -1489,20 +1467,18 @@
       <c r="D34" t="s">
         <v>0</v>
       </c>
-      <c r="E34" t="s">
+      <c r="F34" t="s">
         <v>69</v>
       </c>
-      <c r="F34" t="s">
-        <v>0</v>
-      </c>
-      <c r="I34" t="s">
+      <c r="G34" s="1"/>
+      <c r="J34" t="s">
         <v>71</v>
       </c>
-      <c r="J34">
+      <c r="K34">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>68</v>
       </c>
@@ -1512,14 +1488,14 @@
       <c r="D35" t="s">
         <v>0</v>
       </c>
-      <c r="I35" t="s">
+      <c r="J35" t="s">
         <v>2</v>
       </c>
-      <c r="J35">
+      <c r="K35">
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>67</v>
       </c>
@@ -1529,14 +1505,12 @@
       <c r="D36" t="s">
         <v>0</v>
       </c>
-      <c r="E36" t="s">
+      <c r="F36" t="s">
         <v>66</v>
       </c>
-      <c r="F36" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G36" s="1"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>65</v>
       </c>
@@ -1547,7 +1521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>64</v>
       </c>
@@ -1558,7 +1532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>63</v>
       </c>
@@ -1569,7 +1543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>62</v>
       </c>
@@ -1580,7 +1554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>61</v>
       </c>
@@ -1591,7 +1565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>60</v>
       </c>
@@ -1602,7 +1576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>59</v>
       </c>
@@ -1613,7 +1587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>58</v>
       </c>
@@ -1623,14 +1597,12 @@
       <c r="D44" t="s">
         <v>0</v>
       </c>
-      <c r="E44" t="s">
+      <c r="F44" t="s">
         <v>57</v>
       </c>
-      <c r="F44" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G44" s="1"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>56</v>
       </c>
@@ -1640,14 +1612,12 @@
       <c r="D45" t="s">
         <v>0</v>
       </c>
-      <c r="E45" t="s">
+      <c r="F45" t="s">
         <v>55</v>
       </c>
-      <c r="F45" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G45" s="1"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>54</v>
       </c>
@@ -1657,14 +1627,12 @@
       <c r="D46" t="s">
         <v>0</v>
       </c>
-      <c r="E46" t="s">
+      <c r="F46" t="s">
         <v>53</v>
       </c>
-      <c r="F46" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G46" s="1"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -1674,14 +1642,12 @@
       <c r="D47" t="s">
         <v>0</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" t="s">
         <v>51</v>
       </c>
-      <c r="F47" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="G47" s="1"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>50</v>
       </c>
@@ -1691,14 +1657,12 @@
       <c r="D48" t="s">
         <v>0</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
         <v>49</v>
       </c>
-      <c r="F48" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G48" s="1"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -1709,7 +1673,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>47</v>
       </c>
@@ -1719,14 +1683,12 @@
       <c r="D50" t="s">
         <v>0</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
         <v>46</v>
       </c>
-      <c r="F50" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G50" s="1"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>45</v>
       </c>
@@ -1739,14 +1701,12 @@
       <c r="D51" t="s">
         <v>0</v>
       </c>
-      <c r="E51" t="s">
+      <c r="F51" t="s">
         <v>44</v>
       </c>
-      <c r="F51" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G51" s="1"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>43</v>
       </c>
@@ -1759,14 +1719,12 @@
       <c r="D52" t="s">
         <v>0</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
         <v>42</v>
       </c>
-      <c r="F52" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G52" s="1"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>41</v>
       </c>
@@ -1779,14 +1737,12 @@
       <c r="D53" t="s">
         <v>0</v>
       </c>
-      <c r="E53" t="s">
+      <c r="F53" t="s">
         <v>40</v>
       </c>
-      <c r="F53" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G53" s="1"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>39</v>
       </c>
@@ -1794,7 +1750,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>38</v>
       </c>
@@ -1802,7 +1758,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>37</v>
       </c>
@@ -1810,7 +1766,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>36</v>
       </c>
@@ -1820,17 +1776,15 @@
       <c r="C57" t="s">
         <v>0</v>
       </c>
-      <c r="D57" t="s">
-        <v>0</v>
-      </c>
-      <c r="E57" t="s">
+      <c r="D57" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F57" t="s">
         <v>35</v>
       </c>
-      <c r="F57" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G57" s="1"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>34</v>
       </c>
@@ -1840,17 +1794,15 @@
       <c r="C58" t="s">
         <v>0</v>
       </c>
-      <c r="D58" t="s">
-        <v>0</v>
-      </c>
-      <c r="E58" t="s">
+      <c r="D58" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F58" t="s">
         <v>33</v>
       </c>
-      <c r="F58" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G58" s="1"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>32</v>
       </c>
@@ -1860,53 +1812,51 @@
       <c r="C59" t="s">
         <v>0</v>
       </c>
-      <c r="D59" t="s">
-        <v>0</v>
-      </c>
-      <c r="E59" t="s">
+      <c r="D59" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F59" t="s">
         <v>31</v>
       </c>
-      <c r="F59" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G59" s="1"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>30</v>
       </c>
       <c r="B60">
         <v>60</v>
       </c>
-      <c r="D60" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D60" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>29</v>
       </c>
       <c r="B61">
         <v>61</v>
       </c>
-      <c r="D61" t="s">
-        <v>0</v>
-      </c>
-      <c r="E61" t="s">
+      <c r="D61" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F61" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>28</v>
       </c>
       <c r="B62">
         <v>62</v>
       </c>
-      <c r="D62" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D62" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>27</v>
       </c>
@@ -1914,7 +1864,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>26</v>
       </c>
@@ -1925,7 +1875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>25</v>
       </c>
@@ -1939,7 +1889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>24</v>
       </c>
@@ -1950,7 +1900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>23</v>
       </c>
@@ -1964,7 +1914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -1975,7 +1925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>21</v>
       </c>
@@ -1989,7 +1939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>20</v>
       </c>
@@ -1999,11 +1949,11 @@
       <c r="D70" t="s">
         <v>0</v>
       </c>
-      <c r="E70" s="1" t="s">
+      <c r="F70" s="1" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>19</v>
       </c>
@@ -2014,7 +1964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>126</v>
       </c>
@@ -2027,11 +1977,11 @@
       <c r="D72" t="s">
         <v>0</v>
       </c>
-      <c r="E72" s="1" t="s">
+      <c r="F72" s="1" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>127</v>
       </c>
@@ -2039,7 +1989,7 @@
         <v>72.599999999999994</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>18</v>
       </c>
@@ -2052,11 +2002,17 @@
       <c r="D74" t="s">
         <v>0</v>
       </c>
-      <c r="E74" s="1" t="s">
+      <c r="E74" t="s">
+        <v>135</v>
+      </c>
+      <c r="F74" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="G74" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>17</v>
       </c>
@@ -2069,11 +2025,11 @@
       <c r="D75" t="s">
         <v>0</v>
       </c>
-      <c r="E75" s="1" t="s">
+      <c r="F75" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>16</v>
       </c>
@@ -2084,7 +2040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>15</v>
       </c>
@@ -2095,7 +2051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>14</v>
       </c>
@@ -2106,7 +2062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>13</v>
       </c>
@@ -2117,7 +2073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>12</v>
       </c>
@@ -2229,21 +2185,18 @@
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>133</v>
+        <v>2</v>
       </c>
       <c r="B90">
         <v>92</v>
       </c>
-      <c r="E90" t="s">
+      <c r="F90" t="s">
         <v>2</v>
-      </c>
-      <c r="F90" t="s">
-        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B91">
         <v>93</v>
@@ -2251,16 +2204,13 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>135</v>
+        <v>1</v>
       </c>
       <c r="B92">
         <v>94</v>
       </c>
-      <c r="E92" t="s">
+      <c r="F92" t="s">
         <v>1</v>
-      </c>
-      <c r="F92" t="s">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>